<commit_message>
Final submission: dissertation, slides, user testing results and updated documents
</commit_message>
<xml_diff>
--- a/Capstone_Project/06_Testing_Results_and_Evaluation/Group-3_Requirements_Traceability_Matrix.xlsx
+++ b/Capstone_Project/06_Testing_Results_and_Evaluation/Group-3_Requirements_Traceability_Matrix.xlsx
@@ -884,7 +884,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Confirmation and reminder work in preview mode and an SMTP test email was received on 23 October. The booking emails are still to be checked on the demo laptop</t>
+          <t>Confirmation and reminder work in preview mode, an SMTP test email was received on 23 October and the booking emails arrived on the demonstration laptop</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Scripted journey took 1.8 seconds. The timed test with students is planned for Week 5</t>
+          <t>Scripted journey took 1.8 seconds. The bookings were not timed in the user testing on 28 October (4 students and 2 lecturers)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">

</xml_diff>